<commit_message>
Update Lembar Coding 103 dan Codebook 103 ringkas
</commit_message>
<xml_diff>
--- a/P4 Pengembangan Kebutuhan Perangkat Lunak/A Elisitasi/A4 Coding/Lembar_Coding_Codebook_1_0_3 (Afriansyah).xlsx
+++ b/P4 Pengembangan Kebutuhan Perangkat Lunak/A Elisitasi/A4 Coding/Lembar_Coding_Codebook_1_0_3 (Afriansyah).xlsx
@@ -6479,7 +6479,7 @@
     </ext>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="8" disablePrompts="0">
-        <x14:dataValidation xr:uid="{175B2086-F032-4A75-A813-FFEEB2994A87}" type="list" allowBlank="1" error="Pilih kode dari daftar (lihat sheet Daftar Kode)." errorStyle="stop" errorTitle="Kode tidak sah" imeMode="noControl" operator="between" prompt="Kodekan pihak yang secara eksplisit menjadi subjek tata bahasa norma utama pada kolom “Isi”. Jangan menyimpulkan subjek dari judul BAB." showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{4C3F58AB-9808-43EF-BF23-2169D2C70299}" type="list" allowBlank="1" error="Pilih kode dari daftar (lihat sheet Daftar Kode)." errorStyle="stop" errorTitle="Kode tidak sah" imeMode="noControl" operator="between" prompt="Kodekan pihak yang secara eksplisit menjadi subjek tata bahasa norma utama pada kolom “Isi”. Jangan menyimpulkan subjek dari judul BAB.&#10;Detail lihat Bagian 7.1" promptTitle="" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>'Daftar Kode'!$D$5:$D$13</xm:f>
           </x14:formula1>
@@ -6488,7 +6488,7 @@
           </x14:formula2>
           <xm:sqref>F3:F86</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{2E81922F-C60C-467D-AAB4-7A38B3120AE5}" type="list" allowBlank="1" error="Pilih kode dari daftar (lihat sheet Daftar Kode)." errorStyle="stop" errorTitle="Kode tidak sah" imeMode="noControl" operator="between" prompt="Tentukan dengan Uji Implikasi Bagian 6." showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{5922C192-F2D4-4C66-A9EB-C84BB639CA3E}" type="list" allowBlank="1" error="Pilih kode dari daftar (lihat sheet Daftar Kode)." errorStyle="stop" errorTitle="Kode tidak sah" imeMode="noControl" operator="between" prompt="Tentukan dengan Uji Implikasi Bagian 6.&#10;Detail lainnya lihat Bagian 7.2" promptTitle="" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>'Daftar Kode'!$D$16:$D$18</xm:f>
           </x14:formula1>
@@ -6497,7 +6497,7 @@
           </x14:formula2>
           <xm:sqref>G2:G86</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{2C459CC6-E8CD-4CE9-8F67-7C62AC25D787}" type="list" allowBlank="1" error="Pilih kode dari daftar (lihat sheet Daftar Kode)." errorStyle="stop" errorTitle="Kode tidak sah" imeMode="noControl" operator="between" prompt="Pilih satu tema dominan dari pohon keputusan Bagian 7.3. Pemilihan T99 wajib dijelaskan di V12." showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{5E522288-BC85-4382-B81F-8C02903B5A43}" type="list" allowBlank="1" error="Pilih kode dari daftar (lihat sheet Daftar Kode)." errorStyle="stop" errorTitle="Kode tidak sah" imeMode="noControl" operator="between" prompt="Pilih satu tema dominan dari pohon keputusan Bagian 7.3. Pemilihan T99 wajib dijelaskan di V12." showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>'Daftar Kode'!$D$21:$D$37</xm:f>
           </x14:formula1>
@@ -6506,7 +6506,7 @@
           </x14:formula2>
           <xm:sqref>H2:H86</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{0904CBAE-775E-40B9-A623-71B81123525B}" type="list" allowBlank="1" error="Pilih kode dari daftar (lihat sheet Daftar Kode)." errorStyle="stop" errorTitle="Kode tidak sah" imeMode="noControl" operator="between" prompt="Lihat Bagian 7.4" promptTitle="" showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{18509EE5-9805-474B-92D5-286C3EFA3440}" type="list" allowBlank="1" error="Pilih kode dari daftar (lihat sheet Daftar Kode)." errorStyle="stop" errorTitle="Kode tidak sah" imeMode="noControl" operator="between" prompt="Detail lihat Bagian 7.4" promptTitle="" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>'Daftar Kode'!$D$40:$D$47</xm:f>
           </x14:formula1>
@@ -6515,7 +6515,7 @@
           </x14:formula2>
           <xm:sqref>I2:I86</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{3C7419AB-A381-4E68-B028-35E261E9F56B}" type="list" allowBlank="1" error="Pilih kode dari daftar (lihat sheet Daftar Kode)." errorStyle="stop" errorTitle="Kode tidak sah" imeMode="noControl" operator="between" prompt="Tahap siklus data yang terkait dari awal hingga akhir. Lihat Bagian 7.5" promptTitle="" showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{5A0CD193-FEC6-4215-ADF9-B1DD4467170E}" type="list" allowBlank="1" error="Pilih kode dari daftar (lihat sheet Daftar Kode)." errorStyle="stop" errorTitle="Kode tidak sah" imeMode="noControl" operator="between" prompt="Tahap siklus data yang terkait dari awal hingga akhir.&#10;Detail lihat Bagian 7.5" promptTitle="" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>'Daftar Kode'!$D$50:$D$57</xm:f>
           </x14:formula1>
@@ -6524,7 +6524,7 @@
           </x14:formula2>
           <xm:sqref>J2:J86</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{6BF073CE-56BB-4838-B0B7-22B519CEDAF1}" type="list" allowBlank="1" error="Pilih kode dari daftar (lihat sheet Daftar Kode)." errorStyle="stop" errorTitle="Kode tidak sah" imeMode="noControl" operator="between" prompt="Kandidat jenis kebutuhan SRS diperiksa berurutan K1 -&gt; K2 -&gt; K3 -&gt; K4 -&gt; K5. Lihat Bagian 7.6" promptTitle="" showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{04D8E2A5-939F-4A94-A628-BF202A4F5C84}" type="list" allowBlank="1" error="Pilih kode dari daftar (lihat sheet Daftar Kode)." errorStyle="stop" errorTitle="Kode tidak sah" imeMode="noControl" operator="between" prompt="Kandidat jenis kebutuhan SRS diperiksa berurutan K1 -&gt; K2 -&gt; K3 -&gt; K4 -&gt; K5.&#10;Detail lihat Bagian 7.6" promptTitle="" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>'Daftar Kode'!$D$60:$D$64</xm:f>
           </x14:formula1>
@@ -6533,7 +6533,7 @@
           </x14:formula2>
           <xm:sqref>K2:K86</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{31C63F55-BA88-4F4F-B00F-ACC0C7BDE319}" type="list" allowBlank="1" error="Pilih kode dari daftar (lihat sheet Daftar Kode)." errorStyle="stop" errorTitle="Kode tidak sah" imeMode="noControl" operator="between" prompt="Tema kedua bila unit memuat dua tema (gunakan kode dari Bagian 7.3). T99 tidak digunakan di sini." promptTitle="Opsional" showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{6D8F4892-D741-4689-BFDE-16B14A55AB7E}" type="list" allowBlank="1" error="Pilih kode dari daftar (lihat sheet Daftar Kode)." errorStyle="stop" errorTitle="Kode tidak sah" imeMode="noControl" operator="between" prompt="Tema kedua bila unit memuat dua tema (gunakan kode dari Bagian 7.3). T99 tidak digunakan di sini." promptTitle="Opsional" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>'Daftar Kode'!$D$21:$D$36</xm:f>
           </x14:formula1>
@@ -6542,7 +6542,7 @@
           </x14:formula2>
           <xm:sqref>L2:L86</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{7A994019-6F8E-449B-8E81-B7D06318B958}" type="list" allowBlank="1" error="Pilih kode dari daftar (lihat sheet Daftar Kode)." errorStyle="stop" errorTitle="Kode tidak sah" imeMode="noControl" operator="between" prompt="Kodekan pihak yang secara eksplisit menjadi subjek tata bahasa norma utama pada kolom “Isi”. Jangan menyimpulkan subjek dari judul BAB." promptTitle="" showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{402B7895-FA3E-4444-AAAA-37F5887B5D9F}" type="list" allowBlank="1" error="Pilih kode dari daftar (lihat sheet Daftar Kode)." errorStyle="stop" errorTitle="Kode tidak sah" imeMode="noControl" operator="between" prompt="Kodekan pihak yang secara eksplisit menjadi subjek tata bahasa norma utama pada kolom “Isi”. Jangan menyimpulkan subjek dari judul BAB." promptTitle="" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>'Daftar Kode'!$D$5:$D$13</xm:f>
           </x14:formula1>

</xml_diff>